<commit_message>
Post testing + Android SEAL
Testing has been completed, with one major change being required. The organisations tab has been renamed to join codes, and the delete org button has been moved to its own private section.

SEAL has now been added to both the Android app and the API ready for implementation in the next days.
</commit_message>
<xml_diff>
--- a/Documents/Documentation/API.xlsx
+++ b/Documents/Documentation/API.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccatl\Documents\GitHub\COMP3000\Documents\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFB41852-3AFC-4360-9CDC-00F6E05E6122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E58FC1C-D609-4BBA-89E3-0C34BFF2A08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{BEA67AF9-96E8-423D-96CD-A77CDF9D897A}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BEA67AF9-96E8-423D-96CD-A77CDF9D897A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="160">
   <si>
     <t>Method</t>
   </si>
@@ -574,6 +574,30 @@
   </si>
   <si>
     <t>User</t>
+  </si>
+  <si>
+    <t>/keys/bfv</t>
+  </si>
+  <si>
+    <t>200 OK (JSON: { BFV }), 500 Internal Server Error</t>
+  </si>
+  <si>
+    <t>Returns BFV key for encrypting location data specifcally</t>
+  </si>
+  <si>
+    <t>GPS</t>
+  </si>
+  <si>
+    <t>/gps/update/{deviceId}</t>
+  </si>
+  <si>
+    <t>200 OK , 403 Forbidden</t>
+  </si>
+  <si>
+    <t>Updates the gps location of a given device</t>
+  </si>
+  <si>
+    <t>Body: {signature: string, x: string, y :string}</t>
   </si>
 </sst>
 </file>
@@ -841,7 +865,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -912,14 +936,18 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1255,14 +1283,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D985E0B-1585-4D13-A558-4B9974B4B6FC}">
-  <dimension ref="C4:H52"/>
+  <dimension ref="C4:H55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="39.7109375" customWidth="1"/>
+    <col min="3" max="3" width="38.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30.42578125" customWidth="1"/>
     <col min="6" max="6" width="41.28515625" customWidth="1"/>
-    <col min="7" max="7" width="25.7109375" customWidth="1"/>
+    <col min="7" max="7" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="30.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1357,15 +1385,25 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="3:8">
+    <row r="10" spans="3:8" ht="15.75" thickBot="1">
       <c r="C10" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="13"/>
+      <c r="D10" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="3:8" ht="60">
       <c r="C11" s="23" t="s">
@@ -1427,15 +1465,25 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="3:8">
+    <row r="14" spans="3:8" ht="15.75" thickBot="1">
       <c r="C14" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="13"/>
+      <c r="D14" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="3:8" ht="60">
       <c r="C15" s="23" t="s">
@@ -1517,15 +1565,25 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="3:8">
+    <row r="19" spans="3:8" ht="15.75" thickBot="1">
       <c r="C19" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="13"/>
+      <c r="D19" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="20" spans="3:8" ht="60">
       <c r="C20" s="23" t="s">
@@ -1647,15 +1705,25 @@
         <v>70</v>
       </c>
     </row>
-    <row r="26" spans="3:8">
+    <row r="26" spans="3:8" ht="15.75" thickBot="1">
       <c r="C26" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="13"/>
+      <c r="D26" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="27" spans="3:8" ht="75">
       <c r="C27" s="23" t="s">
@@ -1777,15 +1845,25 @@
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="3:8">
+    <row r="33" spans="3:8" ht="15.75" thickBot="1">
       <c r="C33" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="13"/>
+      <c r="D33" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="34" spans="3:8" ht="45">
       <c r="C34" s="23" t="s">
@@ -1807,334 +1885,424 @@
         <v>89</v>
       </c>
     </row>
-    <row r="35" spans="3:8" ht="60.75" thickBot="1">
-      <c r="C35" s="24" t="s">
+    <row r="35" spans="3:8" ht="60">
+      <c r="C35" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="D35" s="19" t="s">
+      <c r="D35" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E35" s="19" t="s">
+      <c r="E35" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F35" s="19" t="s">
+      <c r="F35" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="G35" s="25">
+      <c r="G35" s="4">
         <v>200400404</v>
       </c>
-      <c r="H35" s="22" t="s">
+      <c r="H35" s="17" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="36" spans="3:8">
-      <c r="C36" s="28" t="s">
+    <row r="36" spans="3:8" ht="30.75" thickBot="1">
+      <c r="C36" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="D36" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="G36" s="30">
+        <v>200500</v>
+      </c>
+      <c r="H36" s="22" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="37" spans="3:8" ht="15.75" thickBot="1">
+      <c r="C37" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="27"/>
-    </row>
-    <row r="37" spans="3:8" ht="45">
-      <c r="C37" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G37" s="4">
-        <v>200400401403</v>
-      </c>
-      <c r="H37" s="17" t="s">
-        <v>97</v>
+      <c r="D37" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="3:8" ht="45">
       <c r="C38" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G38" s="4">
+        <v>200400401403</v>
+      </c>
+      <c r="H38" s="17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="39" spans="3:8" ht="45">
+      <c r="C39" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D39" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E39" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="F39" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="G38" s="4">
+      <c r="G39" s="4">
         <v>201400401403404</v>
       </c>
-      <c r="H38" s="17" t="s">
+      <c r="H39" s="17" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="39" spans="3:8" ht="60.75" thickBot="1">
-      <c r="C39" s="24" t="s">
+    <row r="40" spans="3:8" ht="60.75" thickBot="1">
+      <c r="C40" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="D39" s="19" t="s">
+      <c r="D40" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="E39" s="19" t="s">
+      <c r="E40" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="F39" s="19" t="s">
+      <c r="F40" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="G39" s="25">
+      <c r="G40" s="25">
         <v>200401403404</v>
       </c>
-      <c r="H39" s="22" t="s">
+      <c r="H40" s="22" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="40" spans="3:8">
-      <c r="C40" s="28" t="s">
+    <row r="41" spans="3:8" ht="15.75" thickBot="1">
+      <c r="C41" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="D40" s="26"/>
-      <c r="E40" s="26"/>
-      <c r="F40" s="26"/>
-      <c r="G40" s="26"/>
-      <c r="H40" s="27"/>
-    </row>
-    <row r="41" spans="3:8" ht="60">
-      <c r="C41" s="23" t="s">
+      <c r="D41" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="3:8" ht="60">
+      <c r="C42" s="23" t="s">
         <v>105</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G41" s="4">
-        <v>200401403404</v>
-      </c>
-      <c r="H41" s="17" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="42" spans="3:8" ht="45">
-      <c r="C42" s="23" t="s">
-        <v>108</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>13</v>
       </c>
       <c r="E42" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G42" s="4">
+        <v>200401403404</v>
+      </c>
+      <c r="H42" s="17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="43" spans="3:8" ht="45">
+      <c r="C43" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="F43" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="G42" s="4">
+      <c r="G43" s="4">
         <v>200400401403</v>
       </c>
-      <c r="H42" s="17" t="s">
+      <c r="H43" s="17" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="43" spans="3:8" ht="105">
-      <c r="C43" s="23" t="s">
+    <row r="44" spans="3:8" ht="105">
+      <c r="C44" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="D44" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="E44" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="F44" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G43" s="4">
+      <c r="G44" s="4">
         <v>201401403</v>
       </c>
-      <c r="H43" s="17" t="s">
+      <c r="H44" s="17" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="44" spans="3:8" ht="45.75" thickBot="1">
-      <c r="C44" s="24" t="s">
+    <row r="45" spans="3:8" ht="45.75" thickBot="1">
+      <c r="C45" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="D44" s="19" t="s">
+      <c r="D45" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="E44" s="19" t="s">
+      <c r="E45" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="F44" s="19" t="s">
+      <c r="F45" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="G44" s="25">
+      <c r="G45" s="25">
         <v>200401403409</v>
       </c>
-      <c r="H44" s="22" t="s">
+      <c r="H45" s="22" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="45" spans="3:8">
-      <c r="C45" s="28" t="s">
+    <row r="46" spans="3:8" ht="15.75" thickBot="1">
+      <c r="C46" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="27"/>
-    </row>
-    <row r="46" spans="3:8" ht="45">
-      <c r="C46" s="23" t="s">
+      <c r="D46" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G46" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="3:8" ht="45">
+      <c r="C47" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E47" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F47" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="G46" s="4">
+      <c r="G47" s="4">
         <v>200400401403</v>
       </c>
-      <c r="H46" s="17" t="s">
+      <c r="H47" s="17" t="s">
         <v>122</v>
-      </c>
-    </row>
-    <row r="47" spans="3:8" ht="60">
-      <c r="C47" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="G47" s="4">
-        <v>200401403404</v>
-      </c>
-      <c r="H47" s="17" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="48" spans="3:8" ht="60">
       <c r="C48" s="23" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>127</v>
+        <v>22</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="G48" s="4">
-        <v>200400401403404</v>
+        <v>200401403404</v>
       </c>
       <c r="H48" s="17" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="49" spans="3:8" ht="60">
       <c r="C49" s="23" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E49" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="G49" s="4">
+        <v>200400401403404</v>
+      </c>
+      <c r="H49" s="17" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="50" spans="3:8" ht="60">
+      <c r="C50" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E50" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="F50" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="G49" s="4">
+      <c r="G50" s="4">
         <v>200400401403</v>
       </c>
-      <c r="H49" s="17" t="s">
+      <c r="H50" s="17" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="50" spans="3:8" ht="30">
-      <c r="C50" s="23" t="s">
+    <row r="51" spans="3:8" ht="30">
+      <c r="C51" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="D50" s="1" t="s">
+      <c r="D51" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E50" s="1" t="s">
+      <c r="E51" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="F51" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="G50" s="4">
+      <c r="G51" s="4">
         <v>200400401</v>
       </c>
-      <c r="H50" s="17" t="s">
+      <c r="H51" s="17" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="51" spans="3:8" ht="60">
-      <c r="C51" s="23" t="s">
+    <row r="52" spans="3:8" ht="60">
+      <c r="C52" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="D51" s="1" t="s">
+      <c r="D52" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E51" s="1" t="s">
+      <c r="E52" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="F52" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="G51" s="4">
+      <c r="G52" s="4">
         <v>201400401409500</v>
       </c>
-      <c r="H51" s="17" t="s">
+      <c r="H52" s="17" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="52" spans="3:8" ht="60.75" thickBot="1">
-      <c r="C52" s="24" t="s">
+    <row r="53" spans="3:8" ht="60.75" thickBot="1">
+      <c r="C53" s="24" t="s">
         <v>139</v>
       </c>
-      <c r="D52" s="19" t="s">
+      <c r="D53" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="E52" s="19" t="s">
+      <c r="E53" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="F52" s="19" t="s">
+      <c r="F53" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="G52" s="25">
+      <c r="G53" s="25">
         <v>200401403409500</v>
       </c>
-      <c r="H52" s="22" t="s">
+      <c r="H53" s="22" t="s">
         <v>142</v>
+      </c>
+    </row>
+    <row r="54" spans="3:8" ht="15.75" thickBot="1">
+      <c r="C54" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E54" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F54" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="H54" s="10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="3:8" ht="30">
+      <c r="C55" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="G55" s="4">
+        <v>200403</v>
+      </c>
+      <c r="H55" s="17" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>